<commit_message>
feat: responsive CSS for multi-device
</commit_message>
<xml_diff>
--- a/检修计划数据.xlsx
+++ b/检修计划数据.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>穗水甲线</t>
+          <t>岭深I线</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,42 +488,42 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>待执行</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>500</v>
+        <v>1438</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>广州</t>
+          <t>深圳、惠州</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>220kV</t>
+          <t>500kV</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>模板</t>
+          <t>仿真数据</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>深鹏乙线</t>
+          <t>梅州甲线</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -537,21 +537,21 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>300</v>
+        <v>377</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>深圳</t>
+          <t>梅州、深圳</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -561,59 +561,59 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>模板</t>
+          <t>仿真数据</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>佛肇线</t>
+          <t>揭潮甲线</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>临时检修</t>
+          <t>扩建检修</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>待执行</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>391</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>佛山、肇庆</t>
+          <t>揭阳、汕尾</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>110kV</t>
+          <t>220kV</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>模板</t>
+          <t>仿真数据</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>莞惠甲线</t>
+          <t>深东I线</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -627,11 +627,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>400</v>
+        <v>1113</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -641,62 +641,1187 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>东莞、惠州</t>
+          <t>深圳</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>220kV</t>
+          <t>500kV</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>模板</t>
+          <t>仿真数据</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>湛茂线</t>
+          <t>韶北丙线</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>603</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>韶关、深圳</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>茂湛甲线</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>567</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>茂名、潮州</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>韶赣II线</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>技改检修</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>271</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>韶关</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>中江I线</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>266</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>中山、茂名</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>韶赣I线</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>769</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>韶关、汕头</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>湛海I线</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>临时检修</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1448</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>湛江</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>500kV</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>莞深II线</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>300</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>东莞</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>清韶丙线</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>故障检修</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>52</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>清远、韶关</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>河梅甲线</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>进行中</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>150</v>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="D14" t="n">
+        <v>119</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>河源</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>河惠I线</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>399</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>河源、肇庆</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>江恩乙线</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>118</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>江门</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>东莞甲线</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>临时检修</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>748</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>东莞</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>湛茂甲线</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>扩建检修</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1579</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>湛江</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>500kV</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>汕东I线</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>故障检修</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>188</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>汕头</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>阳云甲线</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>792</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>阳江</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>惠莞I线</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>537</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>惠州</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>阳云丙线</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>阳江、清远</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>中山II线</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>55</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>湛江、茂名</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>中山</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>110kV</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>模板</t>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>惠莞I线</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>技改检修</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>194</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>惠州</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>110kV</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>天广丙线</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1845</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>广州、汕尾</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>500kV</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>清远甲线</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>736</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>清远</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>中山丙线</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>487</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>中山、云浮</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>汕潮乙线</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>技改检修</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>746</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>汕头、阳江</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>汕惠II线</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>技改检修</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>770</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>汕尾、韶关</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>潮汕I线</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>计划检修</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>待执行</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>502</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>潮州、中山</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>汕潮II线</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>故障检修</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>366</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>汕头</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>220kV</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>仿真数据</t>
         </is>
       </c>
     </row>

</xml_diff>